<commit_message>
Update analysis pipeline and generated results
</commit_message>
<xml_diff>
--- a/Analysis/02_CGE_EIPI/2_cge_counterfactual_results.xlsx
+++ b/Analysis/02_CGE_EIPI/2_cge_counterfactual_results.xlsx
@@ -580,13 +580,13 @@
         <v>0.1879200548187051</v>
       </c>
       <c r="Q2" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R2" t="n">
-        <v>16.33065371010141</v>
+        <v>16.96767682052629</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.3465983102620257</v>
+        <v>-0.3951176902621632</v>
       </c>
       <c r="T2" t="n">
         <v>100</v>
@@ -650,13 +650,13 @@
         <v>0.01828309829738651</v>
       </c>
       <c r="Q3" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R3" t="n">
-        <v>16.38755336429825</v>
+        <v>17.03531659487738</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0006164550708251039</v>
+        <v>0.001946199801281802</v>
       </c>
       <c r="T3" t="n">
         <v>100</v>
@@ -720,13 +720,13 @@
         <v>-0.00613649798261512</v>
       </c>
       <c r="Q4" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R4" t="n">
-        <v>16.38695735998724</v>
+        <v>17.03368012339557</v>
       </c>
       <c r="S4" t="n">
-        <v>-0.003020500195547004</v>
+        <v>-0.007660333318897475</v>
       </c>
       <c r="T4" t="n">
         <v>100</v>
@@ -790,13 +790,13 @@
         <v>0.09559609691327986</v>
       </c>
       <c r="Q5" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R5" t="n">
-        <v>16.38658247209441</v>
+        <v>17.03326613215001</v>
       </c>
       <c r="S5" t="n">
-        <v>-0.005308152266032843</v>
+        <v>-0.01009057463754874</v>
       </c>
       <c r="T5" t="n">
         <v>100</v>
@@ -860,13 +860,13 @@
         <v>0.1852365487914815</v>
       </c>
       <c r="Q6" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R6" t="n">
-        <v>16.37981953803016</v>
+        <v>17.02645331982179</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.0465771300344629</v>
+        <v>-0.05008363776153799</v>
       </c>
       <c r="T6" t="n">
         <v>100</v>
@@ -930,13 +930,13 @@
         <v>0.04603756111107495</v>
       </c>
       <c r="Q7" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R7" t="n">
-        <v>16.39714025218297</v>
+        <v>17.03232519512068</v>
       </c>
       <c r="S7" t="n">
-        <v>0.05911784799055923</v>
+        <v>-0.01561413116556806</v>
       </c>
       <c r="T7" t="n">
         <v>100</v>
@@ -1000,13 +1000,13 @@
         <v>0.03483471481113833</v>
       </c>
       <c r="Q8" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R8" t="n">
-        <v>16.38879694872498</v>
+        <v>17.03658505113559</v>
       </c>
       <c r="S8" t="n">
-        <v>0.008205093015889521</v>
+        <v>0.009392383368490673</v>
       </c>
       <c r="T8" t="n">
         <v>100</v>
@@ -1070,13 +1070,13 @@
         <v>0.03897965363301479</v>
       </c>
       <c r="Q9" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R9" t="n">
-        <v>16.38866098229437</v>
+        <v>17.03590997192097</v>
       </c>
       <c r="S9" t="n">
-        <v>0.007375394611487233</v>
+        <v>0.005429484591388718</v>
       </c>
       <c r="T9" t="n">
         <v>100</v>
@@ -1140,13 +1140,13 @@
         <v>0.01661043278833238</v>
       </c>
       <c r="Q10" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R10" t="n">
-        <v>16.3876944948924</v>
+        <v>17.03538661041536</v>
       </c>
       <c r="S10" t="n">
-        <v>0.001477666387859368</v>
+        <v>0.002357210070652354</v>
       </c>
       <c r="T10" t="n">
         <v>100</v>
@@ -1210,13 +1210,13 @@
         <v>0.04871246049247879</v>
       </c>
       <c r="Q11" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R11" t="n">
-        <v>16.39293515755522</v>
+        <v>17.03965508777181</v>
       </c>
       <c r="S11" t="n">
-        <v>0.03345739424989455</v>
+        <v>0.02741433422664738</v>
       </c>
       <c r="T11" t="n">
         <v>100</v>
@@ -1280,13 +1280,13 @@
         <v>0.0695130003018877</v>
       </c>
       <c r="Q12" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R12" t="n">
-        <v>16.39584872907945</v>
+        <v>17.03968806748535</v>
       </c>
       <c r="S12" t="n">
-        <v>0.0512366772235345</v>
+        <v>0.02760793412371342</v>
       </c>
       <c r="T12" t="n">
         <v>100</v>
@@ -1350,13 +1350,13 @@
         <v>0.02042896120074602</v>
       </c>
       <c r="Q13" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R13" t="n">
-        <v>16.38955684531735</v>
+        <v>17.03758680774498</v>
       </c>
       <c r="S13" t="n">
-        <v>0.01284215664521147</v>
+        <v>0.01527296738929809</v>
       </c>
       <c r="T13" t="n">
         <v>100</v>
@@ -1420,13 +1420,13 @@
         <v>0.09771537679263524</v>
       </c>
       <c r="Q14" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R14" t="n">
-        <v>16.39621999101484</v>
+        <v>17.04283396956086</v>
       </c>
       <c r="S14" t="n">
-        <v>0.0535022028684834</v>
+        <v>0.04607523576456057</v>
       </c>
       <c r="T14" t="n">
         <v>100</v>
@@ -1490,13 +1490,13 @@
         <v>0.1295774892219866</v>
       </c>
       <c r="Q15" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R15" t="n">
-        <v>16.39101408934756</v>
+        <v>17.03994177170679</v>
       </c>
       <c r="S15" t="n">
-        <v>0.02173459458925909</v>
+        <v>0.02909724697338812</v>
       </c>
       <c r="T15" t="n">
         <v>100</v>
@@ -1560,13 +1560,13 @@
         <v>0.1226757283933876</v>
       </c>
       <c r="Q16" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R16" t="n">
-        <v>16.40225249151534</v>
+        <v>17.04754420693049</v>
       </c>
       <c r="S16" t="n">
-        <v>0.09031390717878204</v>
+        <v>0.07372561146511762</v>
       </c>
       <c r="T16" t="n">
         <v>100</v>
@@ -1630,13 +1630,13 @@
         <v>0.1431813544838578</v>
       </c>
       <c r="Q17" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R17" t="n">
-        <v>16.40388880208329</v>
+        <v>17.05138437949939</v>
       </c>
       <c r="S17" t="n">
-        <v>0.1002990502852414</v>
+        <v>0.09626846991416807</v>
       </c>
       <c r="T17" t="n">
         <v>100</v>
@@ -1700,13 +1700,13 @@
         <v>0.03091226955722056</v>
       </c>
       <c r="Q18" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R18" t="n">
-        <v>16.39321547062124</v>
+        <v>17.041265604373</v>
       </c>
       <c r="S18" t="n">
-        <v>0.03516792899412285</v>
+        <v>0.03686850513148932</v>
       </c>
       <c r="T18" t="n">
         <v>100</v>
@@ -1770,13 +1770,13 @@
         <v>0.08058230171796413</v>
       </c>
       <c r="Q19" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R19" t="n">
-        <v>16.40446235649073</v>
+        <v>17.04983808612532</v>
       </c>
       <c r="S19" t="n">
-        <v>0.1037990110810122</v>
+        <v>0.08719130683700593</v>
       </c>
       <c r="T19" t="n">
         <v>100</v>
@@ -1840,13 +1840,13 @@
         <v>0.08015224728816542</v>
       </c>
       <c r="Q20" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R20" t="n">
-        <v>16.40932472298705</v>
+        <v>17.05515323597586</v>
       </c>
       <c r="S20" t="n">
-        <v>0.1334702888034321</v>
+        <v>0.1183926834851673</v>
       </c>
       <c r="T20" t="n">
         <v>100</v>
@@ -1910,13 +1910,13 @@
         <v>0.09460429937586783</v>
       </c>
       <c r="Q21" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R21" t="n">
-        <v>16.41864500179638</v>
+        <v>17.0626099266898</v>
       </c>
       <c r="S21" t="n">
-        <v>0.190344771878902</v>
+        <v>0.1621654880263306</v>
       </c>
       <c r="T21" t="n">
         <v>100</v>
@@ -1980,13 +1980,13 @@
         <v>0.0273966663517196</v>
       </c>
       <c r="Q22" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R22" t="n">
-        <v>16.39592133641571</v>
+        <v>17.04204166650922</v>
       </c>
       <c r="S22" t="n">
-        <v>0.05167974387437069</v>
+        <v>0.04142420115053653</v>
       </c>
       <c r="T22" t="n">
         <v>100</v>
@@ -2050,13 +2050,13 @@
         <v>0.0580959704524768</v>
       </c>
       <c r="Q23" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R23" t="n">
-        <v>16.39509079578102</v>
+        <v>17.04163112720789</v>
       </c>
       <c r="S23" t="n">
-        <v>0.04661159406495117</v>
+        <v>0.0390142236842343</v>
       </c>
       <c r="T23" t="n">
         <v>100</v>
@@ -2120,13 +2120,13 @@
         <v>0.04147811380797377</v>
       </c>
       <c r="Q24" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R24" t="n">
-        <v>16.38990280994146</v>
+        <v>17.03723402515688</v>
       </c>
       <c r="S24" t="n">
-        <v>0.01495331228351122</v>
+        <v>0.01320203755371618</v>
       </c>
       <c r="T24" t="n">
         <v>100</v>
@@ -2190,13 +2190,13 @@
         <v>0.2041169216982499</v>
       </c>
       <c r="Q25" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R25" t="n">
-        <v>16.39336017074532</v>
+        <v>17.04777757888794</v>
       </c>
       <c r="S25" t="n">
-        <v>0.03605092240308415</v>
+        <v>0.07509556838980538</v>
       </c>
       <c r="T25" t="n">
         <v>100</v>
@@ -2260,13 +2260,13 @@
         <v>0.011065969760812</v>
       </c>
       <c r="Q26" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R26" t="n">
-        <v>16.38705505418081</v>
+        <v>17.03490181261659</v>
       </c>
       <c r="S26" t="n">
-        <v>-0.002424347776411811</v>
+        <v>-0.0004886849921523742</v>
       </c>
       <c r="T26" t="n">
         <v>100</v>
@@ -2330,13 +2330,13 @@
         <v>0.05678136556034294</v>
       </c>
       <c r="Q27" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R27" t="n">
-        <v>16.38996351414702</v>
+        <v>17.03717166289627</v>
       </c>
       <c r="S27" t="n">
-        <v>0.0153237432954916</v>
+        <v>0.01283595410608849</v>
       </c>
       <c r="T27" t="n">
         <v>100</v>
@@ -2400,13 +2400,13 @@
         <v>0.4071121483645818</v>
       </c>
       <c r="Q28" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R28" t="n">
-        <v>16.38509946781258</v>
+        <v>17.0443470346732</v>
       </c>
       <c r="S28" t="n">
-        <v>-0.01435778518507961</v>
+        <v>0.05495733989913592</v>
       </c>
       <c r="T28" t="n">
         <v>100</v>
@@ -2470,13 +2470,13 @@
         <v>0.1438557735725477</v>
       </c>
       <c r="Q29" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R29" t="n">
-        <v>16.39056450698862</v>
+        <v>17.03839861876047</v>
       </c>
       <c r="S29" t="n">
-        <v>0.01899113972190745</v>
+        <v>0.02003851906211092</v>
       </c>
       <c r="T29" t="n">
         <v>100</v>
@@ -2540,13 +2540,13 @@
         <v>0.3486790936918118</v>
       </c>
       <c r="Q30" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R30" t="n">
-        <v>16.38591337228</v>
+        <v>17.02886738551938</v>
       </c>
       <c r="S30" t="n">
-        <v>-0.009391153091301367</v>
+        <v>-0.03591241489824408</v>
       </c>
       <c r="T30" t="n">
         <v>100</v>
@@ -2610,13 +2610,13 @@
         <v>0.2976064848754095</v>
       </c>
       <c r="Q31" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R31" t="n">
-        <v>16.38308194471803</v>
+        <v>17.0267037470713</v>
       </c>
       <c r="S31" t="n">
-        <v>-0.02666917473073975</v>
+        <v>-0.04861356162921902</v>
       </c>
       <c r="T31" t="n">
         <v>100</v>
@@ -2680,13 +2680,13 @@
         <v>0.3573004884550736</v>
       </c>
       <c r="Q32" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R32" t="n">
-        <v>16.40112872747297</v>
+        <v>17.04613634877665</v>
       </c>
       <c r="S32" t="n">
-        <v>0.08345644075355653</v>
+        <v>0.06546110081904351</v>
       </c>
       <c r="T32" t="n">
         <v>100</v>
@@ -2750,13 +2750,13 @@
         <v>-0.001663398719301727</v>
       </c>
       <c r="Q33" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R33" t="n">
-        <v>16.39027572478958</v>
+        <v>17.03240952351279</v>
       </c>
       <c r="S33" t="n">
-        <v>0.0172289243817706</v>
+        <v>-0.01511910054588435</v>
       </c>
       <c r="T33" t="n">
         <v>100</v>
@@ -2820,13 +2820,13 @@
         <v>0.04029438732864574</v>
       </c>
       <c r="Q34" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R34" t="n">
-        <v>16.38795815932513</v>
+        <v>17.03385622049672</v>
       </c>
       <c r="S34" t="n">
-        <v>0.003086607345899264</v>
+        <v>-0.006626595393466397</v>
       </c>
       <c r="T34" t="n">
         <v>100</v>
@@ -2890,13 +2890,13 @@
         <v>0.1348350346406568</v>
       </c>
       <c r="Q35" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R35" t="n">
-        <v>16.38808964905934</v>
+        <v>17.03347966810697</v>
       </c>
       <c r="S35" t="n">
-        <v>0.003888987920131606</v>
+        <v>-0.00883706043597874</v>
       </c>
       <c r="T35" t="n">
         <v>100</v>
@@ -2960,13 +2960,13 @@
         <v>0.01789608059356288</v>
       </c>
       <c r="Q36" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R36" t="n">
-        <v>16.38728033659022</v>
+        <v>17.03512371462187</v>
       </c>
       <c r="S36" t="n">
-        <v>-0.001049622744756771</v>
+        <v>0.0008139401906950168</v>
       </c>
       <c r="T36" t="n">
         <v>100</v>
@@ -3030,13 +3030,13 @@
         <v>0.1772034951422113</v>
       </c>
       <c r="Q37" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R37" t="n">
-        <v>16.36864310202378</v>
+        <v>17.01857162218917</v>
       </c>
       <c r="S37" t="n">
-        <v>-0.1147783108674245</v>
+        <v>-0.09635134862155696</v>
       </c>
       <c r="T37" t="n">
         <v>100</v>
@@ -3100,13 +3100,13 @@
         <v>0.00673143804365822</v>
       </c>
       <c r="Q38" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R38" t="n">
-        <v>16.38653211877492</v>
+        <v>17.03384415517183</v>
       </c>
       <c r="S38" t="n">
-        <v>-0.005615419792633975</v>
+        <v>-0.006697422135333779</v>
       </c>
       <c r="T38" t="n">
         <v>100</v>
@@ -3170,13 +3170,13 @@
         <v>0.01102129112574966</v>
       </c>
       <c r="Q39" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R39" t="n">
-        <v>16.38629442083743</v>
+        <v>17.03375871227338</v>
       </c>
       <c r="S39" t="n">
-        <v>-0.007065907229692389</v>
+        <v>-0.007198995210650608</v>
       </c>
       <c r="T39" t="n">
         <v>100</v>
@@ -3240,13 +3240,13 @@
         <v>0.02777948206283074</v>
       </c>
       <c r="Q40" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R40" t="n">
-        <v>16.38594341588922</v>
+        <v>17.03405588815441</v>
       </c>
       <c r="S40" t="n">
-        <v>-0.009207820083935477</v>
+        <v>-0.005454491884213056</v>
       </c>
       <c r="T40" t="n">
         <v>100</v>
@@ -3310,13 +3310,13 @@
         <v>0.0753928947740745</v>
       </c>
       <c r="Q41" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R41" t="n">
-        <v>16.3833856028995</v>
+        <v>17.03143527408115</v>
       </c>
       <c r="S41" t="n">
-        <v>-0.02481618272734552</v>
+        <v>-0.0208382099446062</v>
       </c>
       <c r="T41" t="n">
         <v>100</v>
@@ -3380,13 +3380,13 @@
         <v>0.171052380447292</v>
       </c>
       <c r="Q42" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R42" t="n">
-        <v>16.38531425661564</v>
+        <v>17.03556065921794</v>
       </c>
       <c r="S42" t="n">
-        <v>-0.01304709455080364</v>
+        <v>0.003378923925822649</v>
       </c>
       <c r="T42" t="n">
         <v>100</v>
@@ -3450,13 +3450,13 @@
         <v>0.0399489678531709</v>
       </c>
       <c r="Q43" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R43" t="n">
-        <v>16.38406387938453</v>
+        <v>17.03040043015912</v>
       </c>
       <c r="S43" t="n">
-        <v>-0.02067718374917468</v>
+        <v>-0.0269130254985074</v>
       </c>
       <c r="T43" t="n">
         <v>100</v>
@@ -3520,13 +3520,13 @@
         <v>0.009030523174687359</v>
       </c>
       <c r="Q44" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R44" t="n">
-        <v>16.38695186272696</v>
+        <v>17.03459688381016</v>
       </c>
       <c r="S44" t="n">
-        <v>-0.003054045741028504</v>
+        <v>-0.002278700101378356</v>
       </c>
       <c r="T44" t="n">
         <v>100</v>
@@ -3590,13 +3590,13 @@
         <v>0.3177277393241646</v>
       </c>
       <c r="Q45" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R45" t="n">
-        <v>16.36775546915698</v>
+        <v>17.02353876825856</v>
       </c>
       <c r="S45" t="n">
-        <v>-0.1201948505968673</v>
+        <v>-0.06719284891117148</v>
       </c>
       <c r="T45" t="n">
         <v>100</v>
@@ -3660,13 +3660,13 @@
         <v>0.08213897565283053</v>
       </c>
       <c r="Q46" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R46" t="n">
-        <v>16.38541094763529</v>
+        <v>17.03361401986646</v>
       </c>
       <c r="S46" t="n">
-        <v>-0.01245706372952565</v>
+        <v>-0.008048379031123841</v>
       </c>
       <c r="T46" t="n">
         <v>100</v>
@@ -3730,13 +3730,13 @@
         <v>0.05687887101115492</v>
       </c>
       <c r="Q47" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R47" t="n">
-        <v>16.38805920220516</v>
+        <v>17.03597821608347</v>
       </c>
       <c r="S47" t="n">
-        <v>0.003703194219283925</v>
+        <v>0.005830096404442268</v>
       </c>
       <c r="T47" t="n">
         <v>100</v>
@@ -3800,13 +3800,13 @@
         <v>0.002690662810970722</v>
       </c>
       <c r="Q48" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R48" t="n">
-        <v>16.38735559263361</v>
+        <v>17.03496628061724</v>
       </c>
       <c r="S48" t="n">
-        <v>-0.0005903930743400127</v>
+        <v>-0.0001102402771849444</v>
       </c>
       <c r="T48" t="n">
         <v>100</v>
@@ -3870,13 +3870,13 @@
         <v>0.01990000211364723</v>
       </c>
       <c r="Q49" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R49" t="n">
-        <v>16.38681862733288</v>
+        <v>17.03446613991436</v>
       </c>
       <c r="S49" t="n">
-        <v>-0.003867078732887797</v>
+        <v>-0.003046202364150849</v>
       </c>
       <c r="T49" t="n">
         <v>100</v>
@@ -3940,13 +3940,13 @@
         <v>0.01628830313361964</v>
       </c>
       <c r="Q50" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R50" t="n">
-        <v>16.38686256238345</v>
+        <v>17.03426197917083</v>
       </c>
       <c r="S50" t="n">
-        <v>-0.003598976958167983</v>
+        <v>-0.00424468151048282</v>
       </c>
       <c r="T50" t="n">
         <v>100</v>
@@ -4010,13 +4010,13 @@
         <v>0.03118852541845921</v>
       </c>
       <c r="Q51" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R51" t="n">
-        <v>16.385112591243</v>
+        <v>17.03244933783202</v>
       </c>
       <c r="S51" t="n">
-        <v>-0.01427770299693747</v>
+        <v>-0.01488537965273628</v>
       </c>
       <c r="T51" t="n">
         <v>100</v>
@@ -4080,13 +4080,13 @@
         <v>0.03032146434416024</v>
       </c>
       <c r="Q52" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R52" t="n">
-        <v>16.38458206466927</v>
+        <v>17.03341116307566</v>
       </c>
       <c r="S52" t="n">
-        <v>-0.01751509806377641</v>
+        <v>-0.009239203619983625</v>
       </c>
       <c r="T52" t="n">
         <v>100</v>
@@ -4150,13 +4150,13 @@
         <v>0.03214948550430929</v>
       </c>
       <c r="Q53" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R53" t="n">
-        <v>16.38523660558118</v>
+        <v>17.03312671530349</v>
       </c>
       <c r="S53" t="n">
-        <v>-0.01352093900714451</v>
+        <v>-0.0109089894822208</v>
       </c>
       <c r="T53" t="n">
         <v>100</v>
@@ -4220,13 +4220,13 @@
         <v>0.1148216439046681</v>
       </c>
       <c r="Q54" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R54" t="n">
-        <v>16.3879342152127</v>
+        <v>17.03787895207773</v>
       </c>
       <c r="S54" t="n">
-        <v>0.002940494869556345</v>
+        <v>0.01698793415749351</v>
       </c>
       <c r="T54" t="n">
         <v>100</v>
@@ -4290,13 +4290,13 @@
         <v>0.2046128271158935</v>
       </c>
       <c r="Q55" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R55" t="n">
-        <v>16.37115180851544</v>
+        <v>17.02482344878642</v>
       </c>
       <c r="S55" t="n">
-        <v>-0.09946960735973212</v>
+        <v>-0.05965142446419319</v>
       </c>
       <c r="T55" t="n">
         <v>100</v>
@@ -4360,13 +4360,13 @@
         <v>0.05952496954552933</v>
       </c>
       <c r="Q56" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R56" t="n">
-        <v>16.37023368894728</v>
+        <v>17.02178318087735</v>
       </c>
       <c r="S56" t="n">
-        <v>-0.1050721839466054</v>
+        <v>-0.07749862478962509</v>
       </c>
       <c r="T56" t="n">
         <v>100</v>
@@ -4430,13 +4430,13 @@
         <v>0.09237053921623062</v>
       </c>
       <c r="Q57" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R57" t="n">
-        <v>16.37490791210714</v>
+        <v>17.02584820792636</v>
       </c>
       <c r="S57" t="n">
-        <v>-0.07654900009829615</v>
+        <v>-0.0536358093266775</v>
       </c>
       <c r="T57" t="n">
         <v>100</v>
@@ -4500,13 +4500,13 @@
         <v>0.006919731104164557</v>
       </c>
       <c r="Q58" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R58" t="n">
-        <v>16.38662623958533</v>
+        <v>17.03440320799222</v>
       </c>
       <c r="S58" t="n">
-        <v>-0.005041072978767908</v>
+        <v>-0.003415629880049712</v>
       </c>
       <c r="T58" t="n">
         <v>100</v>
@@ -4570,13 +4570,13 @@
         <v>0.02545999485476377</v>
       </c>
       <c r="Q59" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R59" t="n">
-        <v>16.38113388248349</v>
+        <v>17.0301440679995</v>
       </c>
       <c r="S59" t="n">
-        <v>-0.0385566981465825</v>
+        <v>-0.02841794116886209</v>
       </c>
       <c r="T59" t="n">
         <v>100</v>
@@ -4640,13 +4640,13 @@
         <v>0.0134412288636973</v>
       </c>
       <c r="Q60" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R60" t="n">
-        <v>16.38608335850142</v>
+        <v>17.03389382499017</v>
       </c>
       <c r="S60" t="n">
-        <v>-0.008353858105740557</v>
+        <v>-0.006405846779283684</v>
       </c>
       <c r="T60" t="n">
         <v>100</v>
@@ -4710,13 +4710,13 @@
         <v>0.01449149015884511</v>
       </c>
       <c r="Q61" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R61" t="n">
-        <v>16.38552864119903</v>
+        <v>17.03358239478606</v>
       </c>
       <c r="S61" t="n">
-        <v>-0.01173887055783855</v>
+        <v>-0.008234026862855594</v>
       </c>
       <c r="T61" t="n">
         <v>100</v>
@@ -4780,13 +4780,13 @@
         <v>0.007967442147638379</v>
       </c>
       <c r="Q62" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R62" t="n">
-        <v>16.38743584831048</v>
+        <v>17.03517827410338</v>
       </c>
       <c r="S62" t="n">
-        <v>-0.0001006544914652207</v>
+        <v>0.0011342192007438</v>
       </c>
       <c r="T62" t="n">
         <v>100</v>
@@ -4850,13 +4850,13 @@
         <v>0.01243765136264164</v>
       </c>
       <c r="Q63" t="n">
-        <v>16.3874523430173</v>
+        <v>17.03498506003199</v>
       </c>
       <c r="R63" t="n">
-        <v>16.38599693027231</v>
+        <v>17.03395926926841</v>
       </c>
       <c r="S63" t="n">
-        <v>-0.008881263020780319</v>
+        <v>-0.006021671049115598</v>
       </c>
       <c r="T63" t="n">
         <v>100</v>

</xml_diff>